<commit_message>
Rename PI export adjustment label
</commit_message>
<xml_diff>
--- a/assets/system_default_pi_template.xlsx
+++ b/assets/system_default_pi_template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PI Template" sheetId="1" r:id="R3e8fb96f77874275"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PI Template" sheetId="1" r:id="R04cc66c16ea64a65"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -838,7 +838,7 @@
       <x:c r="C19" s="2"/>
       <x:c r="D19" s="2"/>
       <x:c r="E19" s="27" t="str">
-        <x:v>Other Charges / Discount ({{currency}}):</x:v>
+        <x:v>Other Charges ({{currency}}):</x:v>
       </x:c>
       <x:c r="F19" s="27"/>
       <x:c r="G19" s="27"/>

</xml_diff>

<commit_message>
fix: show trade terms in default PI template header
</commit_message>
<xml_diff>
--- a/assets/system_default_pi_template.xlsx
+++ b/assets/system_default_pi_template.xlsx
@@ -715,10 +715,10 @@
     </x:row>
     <x:row r="12" ht="28" customHeight="1">
       <x:c r="A12" s="11" t="str">
-        <x:v>Customer Notes:</x:v>
+        <x:v>Trade Terms:</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
-        <x:v>{{customer_notes}}</x:v>
+        <x:v>{{price_terms}}</x:v>
       </x:c>
       <x:c r="C12" s="14"/>
       <x:c r="D12" s="14"/>

</xml_diff>